<commit_message>
Wire orders to Supabase: save order + address after payment, pre-fill saved address at checkout
</commit_message>
<xml_diff>
--- a/Business/pricing-calculator.xlsx
+++ b/Business/pricing-calculator.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahujadiv\Desktop\Team\Automations\JBG\jewels-by-geetika\business\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahujadiv\Desktop\Team\Automations\Denied\Business\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D80954C4-EE78-4AAE-8105-20C8F406F975}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E89FE95-67C9-433B-9478-E7DC544F0AF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3EA1E2F3-88D9-406C-AEBC-3B66D1D0E7C6}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Product Name</t>
   </si>
@@ -68,58 +68,25 @@
     <t>Net Revenue</t>
   </si>
   <si>
-    <t>Kaveri</t>
+    <t>Ideal Profit</t>
   </si>
   <si>
-    <t>Raahi</t>
+    <t>Signature Oversized</t>
   </si>
   <si>
-    <t>Saanjh</t>
+    <t>Skeleton Acid Wash</t>
   </si>
   <si>
-    <t>Adaa</t>
+    <t>Polo Signature</t>
   </si>
   <si>
-    <t>Ruhani</t>
+    <t>Manual vs Auto</t>
   </si>
   <si>
-    <t>Kanak</t>
+    <t>BaseBall Ottoman Cap</t>
   </si>
   <si>
-    <t>Virasat</t>
-  </si>
-  <si>
-    <t>Sunehri</t>
-  </si>
-  <si>
-    <t>Antara</t>
-  </si>
-  <si>
-    <t>Chandni</t>
-  </si>
-  <si>
-    <t>Rajsi</t>
-  </si>
-  <si>
-    <t>Bella</t>
-  </si>
-  <si>
-    <t>Blossom</t>
-  </si>
-  <si>
-    <t>Grace</t>
-  </si>
-  <si>
-    <t>Ziya</t>
-  </si>
-  <si>
-    <t>Iris</t>
-  </si>
-  <si>
-    <t>Golden Lobster</t>
-  </si>
-  <si>
-    <t>Ideal Profit</t>
+    <t>Snapback Cap</t>
   </si>
 </sst>
 </file>
@@ -991,7 +958,7 @@
   <dimension ref="A1:L18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20.44140625" bestFit="1" customWidth="1"/>
@@ -1033,7 +1000,7 @@
         <v>10</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>2</v>
@@ -1044,767 +1011,689 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B2">
-        <v>71</v>
+        <v>520</v>
       </c>
       <c r="C2">
         <v>50</v>
       </c>
       <c r="D2">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="E2">
         <f t="shared" ref="E2:E17" si="0">B2+C2+D2</f>
-        <v>271</v>
+        <v>670</v>
       </c>
       <c r="F2">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="G2">
-        <f t="shared" ref="G2:G17" si="1">ROUNDUP((E2*F2)/500,0)*500-1</f>
-        <v>999</v>
+        <f>ROUNDUP((E2*F2)/200,0)*200-1</f>
+        <v>1199</v>
       </c>
       <c r="H2">
-        <f t="shared" ref="H2:H18" si="2">G2*2%</f>
-        <v>19.98</v>
+        <f t="shared" ref="H2:H18" si="1">G2*2%</f>
+        <v>23.98</v>
       </c>
       <c r="I2">
-        <f t="shared" ref="I2:I17" si="3">G2-H2</f>
-        <v>979.02</v>
+        <f t="shared" ref="I2:I17" si="2">G2-H2</f>
+        <v>1175.02</v>
       </c>
       <c r="J2">
-        <f t="shared" ref="J2:J17" si="4">I2-E2</f>
-        <v>708.02</v>
+        <f t="shared" ref="J2:J17" si="3">I2-E2</f>
+        <v>505.02</v>
       </c>
       <c r="K2" s="1">
-        <f t="shared" ref="K2:K17" si="5">J2/G2</f>
-        <v>0.70872872872872872</v>
+        <f t="shared" ref="K2:K17" si="4">J2/G2</f>
+        <v>0.42120100083402834</v>
       </c>
       <c r="L2" t="str">
-        <f t="shared" ref="L2:L17" si="6">"₹"&amp;TEXT(G2,"#,##0")</f>
-        <v>₹999</v>
+        <f t="shared" ref="L2:L17" si="5">"₹"&amp;TEXT(G2,"#,##0")</f>
+        <v>₹1,199</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3">
-        <v>110</v>
+        <v>13</v>
       </c>
       <c r="C3">
         <v>50</v>
       </c>
       <c r="D3">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="E3">
         <f t="shared" si="0"/>
-        <v>310</v>
+        <v>150</v>
       </c>
       <c r="F3">
         <v>3</v>
       </c>
       <c r="G3">
+        <f t="shared" ref="G2:G17" si="6">ROUNDUP((E3*F3)/500,0)*500-1</f>
+        <v>499</v>
+      </c>
+      <c r="H3">
         <f t="shared" si="1"/>
-        <v>999</v>
-      </c>
-      <c r="H3">
+        <v>9.98</v>
+      </c>
+      <c r="I3">
         <f t="shared" si="2"/>
-        <v>19.98</v>
-      </c>
-      <c r="I3">
+        <v>489.02</v>
+      </c>
+      <c r="J3">
         <f t="shared" si="3"/>
-        <v>979.02</v>
-      </c>
-      <c r="J3">
+        <v>339.02</v>
+      </c>
+      <c r="K3" s="1">
         <f t="shared" si="4"/>
-        <v>669.02</v>
-      </c>
-      <c r="K3" s="1">
+        <v>0.6793987975951904</v>
+      </c>
+      <c r="L3" t="str">
         <f t="shared" si="5"/>
-        <v>0.66968968968968967</v>
-      </c>
-      <c r="L3" t="str">
-        <f t="shared" si="6"/>
-        <v>₹999</v>
+        <v>₹499</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="B4">
-        <v>145</v>
+        <v>510</v>
       </c>
       <c r="C4">
         <v>50</v>
       </c>
       <c r="D4">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="E4">
         <f t="shared" si="0"/>
-        <v>345</v>
+        <v>660</v>
       </c>
       <c r="F4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G4">
+        <f t="shared" si="6"/>
+        <v>1499</v>
+      </c>
+      <c r="H4">
         <f t="shared" si="1"/>
-        <v>1499</v>
-      </c>
-      <c r="H4">
+        <v>29.98</v>
+      </c>
+      <c r="I4">
         <f t="shared" si="2"/>
-        <v>29.98</v>
-      </c>
-      <c r="I4">
+        <v>1469.02</v>
+      </c>
+      <c r="J4">
         <f t="shared" si="3"/>
-        <v>1469.02</v>
-      </c>
-      <c r="J4">
+        <v>809.02</v>
+      </c>
+      <c r="K4" s="1">
         <f t="shared" si="4"/>
-        <v>1124.02</v>
-      </c>
-      <c r="K4" s="1">
+        <v>0.53970647098065372</v>
+      </c>
+      <c r="L4" t="str">
         <f t="shared" si="5"/>
-        <v>0.74984656437625086</v>
-      </c>
-      <c r="L4" t="str">
-        <f t="shared" si="6"/>
         <v>₹1,499</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B5">
-        <v>425</v>
+        <v>15</v>
       </c>
       <c r="C5">
         <v>50</v>
       </c>
       <c r="D5">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="E5">
         <f t="shared" si="0"/>
-        <v>625</v>
+        <v>150</v>
       </c>
       <c r="F5">
         <v>2</v>
       </c>
       <c r="G5">
+        <f t="shared" si="6"/>
+        <v>499</v>
+      </c>
+      <c r="H5">
         <f t="shared" si="1"/>
-        <v>1499</v>
-      </c>
-      <c r="H5">
+        <v>9.98</v>
+      </c>
+      <c r="I5">
         <f t="shared" si="2"/>
-        <v>29.98</v>
-      </c>
-      <c r="I5">
+        <v>489.02</v>
+      </c>
+      <c r="J5">
         <f t="shared" si="3"/>
-        <v>1469.02</v>
-      </c>
-      <c r="J5">
+        <v>339.02</v>
+      </c>
+      <c r="K5" s="1">
         <f t="shared" si="4"/>
-        <v>844.02</v>
-      </c>
-      <c r="K5" s="1">
+        <v>0.6793987975951904</v>
+      </c>
+      <c r="L5" t="str">
         <f t="shared" si="5"/>
-        <v>0.56305537024683117</v>
-      </c>
-      <c r="L5" t="str">
-        <f t="shared" si="6"/>
-        <v>₹1,499</v>
+        <v>₹499</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>25</v>
-      </c>
-      <c r="B6">
-        <v>380</v>
+        <v>16</v>
       </c>
       <c r="C6">
         <v>50</v>
       </c>
       <c r="D6">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="E6">
         <f t="shared" si="0"/>
-        <v>580</v>
+        <v>150</v>
       </c>
       <c r="F6">
         <v>2.5</v>
       </c>
       <c r="G6">
+        <f t="shared" si="6"/>
+        <v>499</v>
+      </c>
+      <c r="H6">
         <f t="shared" si="1"/>
-        <v>1499</v>
-      </c>
-      <c r="H6">
+        <v>9.98</v>
+      </c>
+      <c r="I6">
         <f t="shared" si="2"/>
-        <v>29.98</v>
-      </c>
-      <c r="I6">
+        <v>489.02</v>
+      </c>
+      <c r="J6">
         <f t="shared" si="3"/>
-        <v>1469.02</v>
-      </c>
-      <c r="J6">
+        <v>339.02</v>
+      </c>
+      <c r="K6" s="1">
         <f t="shared" si="4"/>
-        <v>889.02</v>
-      </c>
-      <c r="K6" s="1">
+        <v>0.6793987975951904</v>
+      </c>
+      <c r="L6" t="str">
         <f t="shared" si="5"/>
-        <v>0.59307538358905931</v>
-      </c>
-      <c r="L6" t="str">
-        <f t="shared" si="6"/>
-        <v>₹1,499</v>
+        <v>₹499</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7">
-        <v>450</v>
+        <v>17</v>
       </c>
       <c r="C7">
         <v>50</v>
       </c>
       <c r="D7">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="E7">
         <f t="shared" si="0"/>
-        <v>650</v>
+        <v>150</v>
       </c>
       <c r="F7">
         <v>3</v>
       </c>
       <c r="G7">
+        <f t="shared" si="6"/>
+        <v>499</v>
+      </c>
+      <c r="H7">
         <f t="shared" si="1"/>
-        <v>1999</v>
-      </c>
-      <c r="H7">
+        <v>9.98</v>
+      </c>
+      <c r="I7">
         <f t="shared" si="2"/>
-        <v>39.980000000000004</v>
-      </c>
-      <c r="I7">
+        <v>489.02</v>
+      </c>
+      <c r="J7">
         <f t="shared" si="3"/>
-        <v>1959.02</v>
-      </c>
-      <c r="J7">
+        <v>339.02</v>
+      </c>
+      <c r="K7" s="1">
         <f t="shared" si="4"/>
-        <v>1309.02</v>
-      </c>
-      <c r="K7" s="1">
+        <v>0.6793987975951904</v>
+      </c>
+      <c r="L7" t="str">
         <f t="shared" si="5"/>
-        <v>0.65483741870935464</v>
-      </c>
-      <c r="L7" t="str">
-        <f t="shared" si="6"/>
-        <v>₹1,999</v>
+        <v>₹499</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>22</v>
-      </c>
-      <c r="B8">
-        <v>456</v>
-      </c>
       <c r="C8">
         <v>50</v>
       </c>
       <c r="D8">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="E8">
         <f t="shared" si="0"/>
-        <v>656</v>
+        <v>150</v>
       </c>
       <c r="F8">
         <v>3</v>
       </c>
       <c r="G8">
+        <f t="shared" si="6"/>
+        <v>499</v>
+      </c>
+      <c r="H8">
         <f t="shared" si="1"/>
-        <v>1999</v>
-      </c>
-      <c r="H8">
+        <v>9.98</v>
+      </c>
+      <c r="I8">
         <f t="shared" si="2"/>
-        <v>39.980000000000004</v>
-      </c>
-      <c r="I8">
+        <v>489.02</v>
+      </c>
+      <c r="J8">
         <f t="shared" si="3"/>
-        <v>1959.02</v>
-      </c>
-      <c r="J8">
+        <v>339.02</v>
+      </c>
+      <c r="K8" s="1">
         <f t="shared" si="4"/>
-        <v>1303.02</v>
-      </c>
-      <c r="K8" s="1">
+        <v>0.6793987975951904</v>
+      </c>
+      <c r="L8" t="str">
         <f t="shared" si="5"/>
-        <v>0.65183591795897944</v>
-      </c>
-      <c r="L8" t="str">
-        <f t="shared" si="6"/>
-        <v>₹1,999</v>
+        <v>₹499</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>26</v>
-      </c>
-      <c r="B9">
-        <v>480</v>
-      </c>
       <c r="C9">
         <v>50</v>
       </c>
       <c r="D9">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="E9">
         <f t="shared" si="0"/>
-        <v>680</v>
+        <v>150</v>
       </c>
       <c r="F9">
         <v>2.5</v>
       </c>
       <c r="G9">
+        <f t="shared" si="6"/>
+        <v>499</v>
+      </c>
+      <c r="H9">
         <f t="shared" si="1"/>
-        <v>1999</v>
-      </c>
-      <c r="H9">
+        <v>9.98</v>
+      </c>
+      <c r="I9">
         <f t="shared" si="2"/>
-        <v>39.980000000000004</v>
-      </c>
-      <c r="I9">
+        <v>489.02</v>
+      </c>
+      <c r="J9">
         <f t="shared" si="3"/>
-        <v>1959.02</v>
-      </c>
-      <c r="J9">
+        <v>339.02</v>
+      </c>
+      <c r="K9" s="1">
         <f t="shared" si="4"/>
-        <v>1279.02</v>
-      </c>
-      <c r="K9" s="1">
+        <v>0.6793987975951904</v>
+      </c>
+      <c r="L9" t="str">
         <f t="shared" si="5"/>
-        <v>0.63982991495747876</v>
-      </c>
-      <c r="L9" t="str">
-        <f t="shared" si="6"/>
-        <v>₹1,999</v>
+        <v>₹499</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10">
-        <v>472</v>
-      </c>
       <c r="C10">
         <v>50</v>
       </c>
       <c r="D10">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="E10">
         <f t="shared" si="0"/>
-        <v>672</v>
+        <v>150</v>
       </c>
       <c r="F10">
         <v>3</v>
       </c>
       <c r="G10">
+        <f t="shared" si="6"/>
+        <v>499</v>
+      </c>
+      <c r="H10">
         <f t="shared" si="1"/>
-        <v>2499</v>
-      </c>
-      <c r="H10">
+        <v>9.98</v>
+      </c>
+      <c r="I10">
         <f t="shared" si="2"/>
-        <v>49.980000000000004</v>
-      </c>
-      <c r="I10">
+        <v>489.02</v>
+      </c>
+      <c r="J10">
         <f t="shared" si="3"/>
-        <v>2449.02</v>
-      </c>
-      <c r="J10">
+        <v>339.02</v>
+      </c>
+      <c r="K10" s="1">
         <f t="shared" si="4"/>
-        <v>1777.02</v>
-      </c>
-      <c r="K10" s="1">
+        <v>0.6793987975951904</v>
+      </c>
+      <c r="L10" t="str">
         <f t="shared" si="5"/>
-        <v>0.71109243697478985</v>
-      </c>
-      <c r="L10" t="str">
-        <f t="shared" si="6"/>
-        <v>₹2,499</v>
+        <v>₹499</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>21</v>
-      </c>
-      <c r="B11">
-        <v>654</v>
-      </c>
       <c r="C11">
         <v>50</v>
       </c>
       <c r="D11">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="E11">
         <f t="shared" si="0"/>
-        <v>854</v>
+        <v>150</v>
       </c>
       <c r="F11">
         <v>3</v>
       </c>
       <c r="G11">
+        <f t="shared" si="6"/>
+        <v>499</v>
+      </c>
+      <c r="H11">
         <f t="shared" si="1"/>
-        <v>2999</v>
-      </c>
-      <c r="H11">
+        <v>9.98</v>
+      </c>
+      <c r="I11">
         <f t="shared" si="2"/>
-        <v>59.980000000000004</v>
-      </c>
-      <c r="I11">
+        <v>489.02</v>
+      </c>
+      <c r="J11">
         <f t="shared" si="3"/>
-        <v>2939.02</v>
-      </c>
-      <c r="J11">
+        <v>339.02</v>
+      </c>
+      <c r="K11" s="1">
         <f t="shared" si="4"/>
-        <v>2085.02</v>
-      </c>
-      <c r="K11" s="1">
+        <v>0.6793987975951904</v>
+      </c>
+      <c r="L11" t="str">
         <f t="shared" si="5"/>
-        <v>0.69523841280426812</v>
-      </c>
-      <c r="L11" t="str">
-        <f t="shared" si="6"/>
-        <v>₹2,999</v>
+        <v>₹499</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>14</v>
-      </c>
-      <c r="B12">
-        <v>1134</v>
-      </c>
       <c r="C12">
         <v>30</v>
       </c>
       <c r="D12">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="E12">
         <f t="shared" si="0"/>
-        <v>1314</v>
+        <v>130</v>
       </c>
       <c r="F12">
         <v>3</v>
       </c>
       <c r="G12">
+        <f t="shared" si="6"/>
+        <v>499</v>
+      </c>
+      <c r="H12">
         <f t="shared" si="1"/>
-        <v>3999</v>
-      </c>
-      <c r="H12">
+        <v>9.98</v>
+      </c>
+      <c r="I12">
         <f t="shared" si="2"/>
-        <v>79.98</v>
-      </c>
-      <c r="I12">
+        <v>489.02</v>
+      </c>
+      <c r="J12">
         <f t="shared" si="3"/>
-        <v>3919.02</v>
-      </c>
-      <c r="J12">
+        <v>359.02</v>
+      </c>
+      <c r="K12" s="1">
         <f t="shared" si="4"/>
-        <v>2605.02</v>
-      </c>
-      <c r="K12" s="1">
+        <v>0.71947895791583161</v>
+      </c>
+      <c r="L12" t="str">
         <f t="shared" si="5"/>
-        <v>0.65141785446361589</v>
-      </c>
-      <c r="L12" t="str">
-        <f t="shared" si="6"/>
-        <v>₹3,999</v>
+        <v>₹499</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>15</v>
-      </c>
-      <c r="B13">
-        <v>2100</v>
-      </c>
       <c r="C13">
         <v>30</v>
       </c>
       <c r="D13">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="E13">
         <f t="shared" si="0"/>
-        <v>2280</v>
+        <v>130</v>
       </c>
       <c r="F13">
         <v>1.75</v>
       </c>
       <c r="G13">
+        <f t="shared" si="6"/>
+        <v>499</v>
+      </c>
+      <c r="H13">
         <f t="shared" si="1"/>
-        <v>3999</v>
-      </c>
-      <c r="H13">
+        <v>9.98</v>
+      </c>
+      <c r="I13">
         <f t="shared" si="2"/>
-        <v>79.98</v>
-      </c>
-      <c r="I13">
+        <v>489.02</v>
+      </c>
+      <c r="J13">
         <f t="shared" si="3"/>
-        <v>3919.02</v>
-      </c>
-      <c r="J13">
+        <v>359.02</v>
+      </c>
+      <c r="K13" s="1">
         <f t="shared" si="4"/>
-        <v>1639.02</v>
-      </c>
-      <c r="K13" s="1">
+        <v>0.71947895791583161</v>
+      </c>
+      <c r="L13" t="str">
         <f t="shared" si="5"/>
-        <v>0.4098574643660915</v>
-      </c>
-      <c r="L13" t="str">
-        <f t="shared" si="6"/>
-        <v>₹3,999</v>
+        <v>₹499</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>19</v>
-      </c>
-      <c r="B14">
-        <v>1070</v>
-      </c>
       <c r="C14">
         <v>50</v>
       </c>
       <c r="D14">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="E14">
         <f t="shared" si="0"/>
-        <v>1270</v>
+        <v>150</v>
       </c>
       <c r="F14">
         <v>3</v>
       </c>
       <c r="G14">
+        <f t="shared" si="6"/>
+        <v>499</v>
+      </c>
+      <c r="H14">
         <f t="shared" si="1"/>
-        <v>3999</v>
-      </c>
-      <c r="H14">
+        <v>9.98</v>
+      </c>
+      <c r="I14">
         <f t="shared" si="2"/>
-        <v>79.98</v>
-      </c>
-      <c r="I14">
+        <v>489.02</v>
+      </c>
+      <c r="J14">
         <f t="shared" si="3"/>
-        <v>3919.02</v>
-      </c>
-      <c r="J14">
+        <v>339.02</v>
+      </c>
+      <c r="K14" s="1">
         <f t="shared" si="4"/>
-        <v>2649.02</v>
-      </c>
-      <c r="K14" s="1">
+        <v>0.6793987975951904</v>
+      </c>
+      <c r="L14" t="str">
         <f t="shared" si="5"/>
-        <v>0.66242060515128787</v>
-      </c>
-      <c r="L14" t="str">
-        <f t="shared" si="6"/>
-        <v>₹3,999</v>
+        <v>₹499</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>20</v>
-      </c>
-      <c r="B15">
-        <v>1069</v>
-      </c>
       <c r="C15">
         <v>50</v>
       </c>
       <c r="D15">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="E15">
         <f t="shared" si="0"/>
-        <v>1269</v>
+        <v>150</v>
       </c>
       <c r="F15">
         <v>3</v>
       </c>
       <c r="G15">
+        <f t="shared" si="6"/>
+        <v>499</v>
+      </c>
+      <c r="H15">
         <f t="shared" si="1"/>
-        <v>3999</v>
-      </c>
-      <c r="H15">
+        <v>9.98</v>
+      </c>
+      <c r="I15">
         <f t="shared" si="2"/>
-        <v>79.98</v>
-      </c>
-      <c r="I15">
+        <v>489.02</v>
+      </c>
+      <c r="J15">
         <f t="shared" si="3"/>
-        <v>3919.02</v>
-      </c>
-      <c r="J15">
+        <v>339.02</v>
+      </c>
+      <c r="K15" s="1">
         <f t="shared" si="4"/>
-        <v>2650.02</v>
-      </c>
-      <c r="K15" s="1">
+        <v>0.6793987975951904</v>
+      </c>
+      <c r="L15" t="str">
         <f t="shared" si="5"/>
-        <v>0.66267066766691674</v>
-      </c>
-      <c r="L15" t="str">
-        <f t="shared" si="6"/>
-        <v>₹3,999</v>
+        <v>₹499</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>12</v>
-      </c>
-      <c r="B16">
-        <v>1240</v>
-      </c>
       <c r="C16">
         <v>50</v>
       </c>
       <c r="D16">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="E16">
         <f t="shared" si="0"/>
-        <v>1440</v>
+        <v>150</v>
       </c>
       <c r="F16">
         <v>3</v>
       </c>
       <c r="G16">
+        <f t="shared" si="6"/>
+        <v>499</v>
+      </c>
+      <c r="H16">
         <f t="shared" si="1"/>
-        <v>4499</v>
-      </c>
-      <c r="H16">
+        <v>9.98</v>
+      </c>
+      <c r="I16">
         <f t="shared" si="2"/>
-        <v>89.98</v>
-      </c>
-      <c r="I16">
+        <v>489.02</v>
+      </c>
+      <c r="J16">
         <f t="shared" si="3"/>
-        <v>4409.0200000000004</v>
-      </c>
-      <c r="J16">
+        <v>339.02</v>
+      </c>
+      <c r="K16" s="1">
         <f t="shared" si="4"/>
-        <v>2969.0200000000004</v>
-      </c>
-      <c r="K16" s="1">
+        <v>0.6793987975951904</v>
+      </c>
+      <c r="L16" t="str">
         <f t="shared" si="5"/>
-        <v>0.65992887308290737</v>
-      </c>
-      <c r="L16" t="str">
-        <f t="shared" si="6"/>
-        <v>₹4,499</v>
+        <v>₹499</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>13</v>
-      </c>
-      <c r="B17">
-        <v>1495</v>
-      </c>
+    <row r="17" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C17">
         <v>50</v>
       </c>
       <c r="D17">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="E17">
         <f t="shared" si="0"/>
-        <v>1695</v>
+        <v>150</v>
       </c>
       <c r="F17">
         <v>3</v>
       </c>
       <c r="G17">
+        <f t="shared" si="6"/>
+        <v>499</v>
+      </c>
+      <c r="H17">
         <f t="shared" si="1"/>
-        <v>5499</v>
-      </c>
-      <c r="H17">
+        <v>9.98</v>
+      </c>
+      <c r="I17">
         <f t="shared" si="2"/>
-        <v>109.98</v>
-      </c>
-      <c r="I17">
+        <v>489.02</v>
+      </c>
+      <c r="J17">
         <f t="shared" si="3"/>
-        <v>5389.02</v>
-      </c>
-      <c r="J17">
+        <v>339.02</v>
+      </c>
+      <c r="K17" s="1">
         <f t="shared" si="4"/>
-        <v>3694.0200000000004</v>
-      </c>
-      <c r="K17" s="1">
+        <v>0.6793987975951904</v>
+      </c>
+      <c r="L17" t="str">
         <f t="shared" si="5"/>
-        <v>0.67176213857064926</v>
-      </c>
-      <c r="L17" t="str">
-        <f t="shared" si="6"/>
-        <v>₹5,499</v>
+        <v>₹499</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>27</v>
-      </c>
-      <c r="B18">
-        <v>768</v>
-      </c>
+    <row r="18" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C18">
         <v>50</v>
       </c>
       <c r="D18">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="E18">
         <f t="shared" ref="E18" si="7">B18+C18+D18</f>
-        <v>968</v>
+        <v>150</v>
       </c>
       <c r="F18">
         <v>3</v>
       </c>
       <c r="G18">
         <f t="shared" ref="G18" si="8">ROUNDUP((E18*F18)/500,0)*500-1</f>
-        <v>2999</v>
+        <v>499</v>
       </c>
       <c r="H18">
-        <f t="shared" si="2"/>
-        <v>59.980000000000004</v>
+        <f t="shared" si="1"/>
+        <v>9.98</v>
       </c>
       <c r="I18">
         <f t="shared" ref="I18" si="9">G18-H18</f>
-        <v>2939.02</v>
+        <v>489.02</v>
       </c>
       <c r="J18">
         <f t="shared" ref="J18" si="10">I18-E18</f>
-        <v>1971.02</v>
+        <v>339.02</v>
       </c>
       <c r="K18" s="1">
         <f t="shared" ref="K18" si="11">J18/G18</f>
-        <v>0.65722574191397132</v>
+        <v>0.6793987975951904</v>
       </c>
       <c r="L18" t="str">
         <f t="shared" ref="L18" si="12">"₹"&amp;TEXT(G18,"#,##0")</f>
-        <v>₹2,999</v>
+        <v>₹499</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update all products: new paths, updated prices, new colors (Polo 6 colors, Supima 3 colors), renamed designs
</commit_message>
<xml_diff>
--- a/Business/pricing-calculator.xlsx
+++ b/Business/pricing-calculator.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahujadiv\Desktop\Team\Automations\Denied\Business\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E89FE95-67C9-433B-9478-E7DC544F0AF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FB2E83D-85D2-4724-BB8F-5A665699CF3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3EA1E2F3-88D9-406C-AEBC-3B66D1D0E7C6}"/>
+    <workbookView xWindow="32856" yWindow="912" windowWidth="34560" windowHeight="18600" xr2:uid="{3EA1E2F3-88D9-406C-AEBC-3B66D1D0E7C6}"/>
   </bookViews>
   <sheets>
     <sheet name="pricing-calculator" sheetId="1" r:id="rId1"/>
@@ -1058,6 +1058,9 @@
       <c r="A3" t="s">
         <v>13</v>
       </c>
+      <c r="B3">
+        <v>710</v>
+      </c>
       <c r="C3">
         <v>50</v>
       </c>
@@ -1066,34 +1069,34 @@
       </c>
       <c r="E3">
         <f t="shared" si="0"/>
-        <v>150</v>
+        <v>860</v>
       </c>
       <c r="F3">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="G3">
-        <f t="shared" ref="G2:G17" si="6">ROUNDUP((E3*F3)/500,0)*500-1</f>
-        <v>499</v>
+        <f t="shared" ref="G3:G17" si="6">ROUNDUP((E3*F3)/500,0)*500-1</f>
+        <v>1499</v>
       </c>
       <c r="H3">
         <f t="shared" si="1"/>
-        <v>9.98</v>
+        <v>29.98</v>
       </c>
       <c r="I3">
         <f t="shared" si="2"/>
-        <v>489.02</v>
+        <v>1469.02</v>
       </c>
       <c r="J3">
         <f t="shared" si="3"/>
-        <v>339.02</v>
+        <v>609.02</v>
       </c>
       <c r="K3" s="1">
         <f t="shared" si="4"/>
-        <v>0.6793987975951904</v>
+        <v>0.40628418945963973</v>
       </c>
       <c r="L3" t="str">
         <f t="shared" si="5"/>
-        <v>₹499</v>
+        <v>₹1,499</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
@@ -1101,7 +1104,7 @@
         <v>14</v>
       </c>
       <c r="B4">
-        <v>510</v>
+        <v>540</v>
       </c>
       <c r="C4">
         <v>50</v>
@@ -1111,10 +1114,10 @@
       </c>
       <c r="E4">
         <f t="shared" si="0"/>
-        <v>660</v>
+        <v>690</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="G4">
         <f t="shared" si="6"/>
@@ -1130,11 +1133,11 @@
       </c>
       <c r="J4">
         <f t="shared" si="3"/>
-        <v>809.02</v>
+        <v>779.02</v>
       </c>
       <c r="K4" s="1">
         <f t="shared" si="4"/>
-        <v>0.53970647098065372</v>
+        <v>0.51969312875250162</v>
       </c>
       <c r="L4" t="str">
         <f t="shared" si="5"/>
@@ -1145,6 +1148,9 @@
       <c r="A5" t="s">
         <v>15</v>
       </c>
+      <c r="B5">
+        <v>745</v>
+      </c>
       <c r="C5">
         <v>50</v>
       </c>
@@ -1153,40 +1159,43 @@
       </c>
       <c r="E5">
         <f t="shared" si="0"/>
-        <v>150</v>
+        <v>895</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="G5">
         <f t="shared" si="6"/>
-        <v>499</v>
+        <v>1499</v>
       </c>
       <c r="H5">
         <f t="shared" si="1"/>
-        <v>9.98</v>
+        <v>29.98</v>
       </c>
       <c r="I5">
         <f t="shared" si="2"/>
-        <v>489.02</v>
+        <v>1469.02</v>
       </c>
       <c r="J5">
         <f t="shared" si="3"/>
-        <v>339.02</v>
+        <v>574.02</v>
       </c>
       <c r="K5" s="1">
         <f t="shared" si="4"/>
-        <v>0.6793987975951904</v>
+        <v>0.38293529019346229</v>
       </c>
       <c r="L5" t="str">
         <f t="shared" si="5"/>
-        <v>₹499</v>
+        <v>₹1,499</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>16</v>
       </c>
+      <c r="B6">
+        <v>465</v>
+      </c>
       <c r="C6">
         <v>50</v>
       </c>
@@ -1195,40 +1204,43 @@
       </c>
       <c r="E6">
         <f t="shared" si="0"/>
-        <v>150</v>
+        <v>615</v>
       </c>
       <c r="F6">
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c r="G6">
         <f t="shared" si="6"/>
-        <v>499</v>
+        <v>999</v>
       </c>
       <c r="H6">
         <f t="shared" si="1"/>
-        <v>9.98</v>
+        <v>19.98</v>
       </c>
       <c r="I6">
         <f t="shared" si="2"/>
-        <v>489.02</v>
+        <v>979.02</v>
       </c>
       <c r="J6">
         <f t="shared" si="3"/>
-        <v>339.02</v>
+        <v>364.02</v>
       </c>
       <c r="K6" s="1">
         <f t="shared" si="4"/>
-        <v>0.6793987975951904</v>
+        <v>0.36438438438438436</v>
       </c>
       <c r="L6" t="str">
         <f t="shared" si="5"/>
-        <v>₹499</v>
+        <v>₹999</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>17</v>
       </c>
+      <c r="B7">
+        <v>465</v>
+      </c>
       <c r="C7">
         <v>50</v>
       </c>
@@ -1237,34 +1249,34 @@
       </c>
       <c r="E7">
         <f t="shared" si="0"/>
-        <v>150</v>
+        <v>615</v>
       </c>
       <c r="F7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G7">
         <f t="shared" si="6"/>
-        <v>499</v>
+        <v>999</v>
       </c>
       <c r="H7">
         <f t="shared" si="1"/>
-        <v>9.98</v>
+        <v>19.98</v>
       </c>
       <c r="I7">
         <f t="shared" si="2"/>
-        <v>489.02</v>
+        <v>979.02</v>
       </c>
       <c r="J7">
         <f t="shared" si="3"/>
-        <v>339.02</v>
+        <v>364.02</v>
       </c>
       <c r="K7" s="1">
         <f t="shared" si="4"/>
-        <v>0.6793987975951904</v>
+        <v>0.36438438438438436</v>
       </c>
       <c r="L7" t="str">
         <f t="shared" si="5"/>
-        <v>₹499</v>
+        <v>₹999</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Harden launch checkout and complete site readiness
</commit_message>
<xml_diff>
--- a/Business/pricing-calculator.xlsx
+++ b/Business/pricing-calculator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahujadiv\Desktop\Team\Automations\Denied\Business\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FB2E83D-85D2-4724-BB8F-5A665699CF3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5A371CC-2395-473A-B446-B32000AEDA02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32856" yWindow="912" windowWidth="34560" windowHeight="18600" xr2:uid="{3EA1E2F3-88D9-406C-AEBC-3B66D1D0E7C6}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="46296" windowHeight="25416" xr2:uid="{3EA1E2F3-88D9-406C-AEBC-3B66D1D0E7C6}"/>
   </bookViews>
   <sheets>
     <sheet name="pricing-calculator" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Product Name</t>
   </si>
@@ -87,6 +87,9 @@
   </si>
   <si>
     <t>Snapback Cap</t>
+  </si>
+  <si>
+    <t>Unique</t>
   </si>
 </sst>
 </file>
@@ -1075,28 +1078,28 @@
         <v>1.5</v>
       </c>
       <c r="G3">
-        <f t="shared" ref="G3:G17" si="6">ROUNDUP((E3*F3)/500,0)*500-1</f>
-        <v>1499</v>
+        <f t="shared" ref="G3:G18" si="6">ROUNDUP((E3*F3)/200,0)*200-1</f>
+        <v>1399</v>
       </c>
       <c r="H3">
         <f t="shared" si="1"/>
-        <v>29.98</v>
+        <v>27.98</v>
       </c>
       <c r="I3">
         <f t="shared" si="2"/>
-        <v>1469.02</v>
+        <v>1371.02</v>
       </c>
       <c r="J3">
         <f t="shared" si="3"/>
-        <v>609.02</v>
+        <v>511.02</v>
       </c>
       <c r="K3" s="1">
         <f t="shared" si="4"/>
-        <v>0.40628418945963973</v>
+        <v>0.36527519656897783</v>
       </c>
       <c r="L3" t="str">
         <f t="shared" si="5"/>
-        <v>₹1,499</v>
+        <v>₹1,399</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
@@ -1121,27 +1124,27 @@
       </c>
       <c r="G4">
         <f t="shared" si="6"/>
-        <v>1499</v>
+        <v>1199</v>
       </c>
       <c r="H4">
         <f t="shared" si="1"/>
-        <v>29.98</v>
+        <v>23.98</v>
       </c>
       <c r="I4">
         <f t="shared" si="2"/>
-        <v>1469.02</v>
+        <v>1175.02</v>
       </c>
       <c r="J4">
         <f t="shared" si="3"/>
-        <v>779.02</v>
+        <v>485.02</v>
       </c>
       <c r="K4" s="1">
         <f t="shared" si="4"/>
-        <v>0.51969312875250162</v>
+        <v>0.40452043369474561</v>
       </c>
       <c r="L4" t="str">
         <f t="shared" si="5"/>
-        <v>₹1,499</v>
+        <v>₹1,199</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
@@ -1166,27 +1169,27 @@
       </c>
       <c r="G5">
         <f t="shared" si="6"/>
-        <v>1499</v>
+        <v>1399</v>
       </c>
       <c r="H5">
         <f t="shared" si="1"/>
-        <v>29.98</v>
+        <v>27.98</v>
       </c>
       <c r="I5">
         <f t="shared" si="2"/>
-        <v>1469.02</v>
+        <v>1371.02</v>
       </c>
       <c r="J5">
         <f t="shared" si="3"/>
-        <v>574.02</v>
+        <v>476.02</v>
       </c>
       <c r="K5" s="1">
         <f t="shared" si="4"/>
-        <v>0.38293529019346229</v>
+        <v>0.34025732666190134</v>
       </c>
       <c r="L5" t="str">
         <f t="shared" si="5"/>
-        <v>₹1,499</v>
+        <v>₹1,399</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
@@ -1211,27 +1214,27 @@
       </c>
       <c r="G6">
         <f t="shared" si="6"/>
-        <v>999</v>
+        <v>799</v>
       </c>
       <c r="H6">
         <f t="shared" si="1"/>
-        <v>19.98</v>
+        <v>15.98</v>
       </c>
       <c r="I6">
         <f t="shared" si="2"/>
-        <v>979.02</v>
+        <v>783.02</v>
       </c>
       <c r="J6">
         <f t="shared" si="3"/>
-        <v>364.02</v>
+        <v>168.01999999999998</v>
       </c>
       <c r="K6" s="1">
         <f t="shared" si="4"/>
-        <v>0.36438438438438436</v>
+        <v>0.21028785982478096</v>
       </c>
       <c r="L6" t="str">
         <f t="shared" si="5"/>
-        <v>₹999</v>
+        <v>₹799</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
@@ -1256,30 +1259,36 @@
       </c>
       <c r="G7">
         <f t="shared" si="6"/>
-        <v>999</v>
+        <v>799</v>
       </c>
       <c r="H7">
         <f t="shared" si="1"/>
-        <v>19.98</v>
+        <v>15.98</v>
       </c>
       <c r="I7">
         <f t="shared" si="2"/>
-        <v>979.02</v>
+        <v>783.02</v>
       </c>
       <c r="J7">
         <f t="shared" si="3"/>
-        <v>364.02</v>
+        <v>168.01999999999998</v>
       </c>
       <c r="K7" s="1">
         <f t="shared" si="4"/>
-        <v>0.36438438438438436</v>
+        <v>0.21028785982478096</v>
       </c>
       <c r="L7" t="str">
         <f t="shared" si="5"/>
-        <v>₹999</v>
+        <v>₹799</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8">
+        <v>570</v>
+      </c>
       <c r="C8">
         <v>50</v>
       </c>
@@ -1288,34 +1297,34 @@
       </c>
       <c r="E8">
         <f t="shared" si="0"/>
-        <v>150</v>
+        <v>720</v>
       </c>
       <c r="F8">
-        <v>3</v>
+        <v>1.8</v>
       </c>
       <c r="G8">
         <f t="shared" si="6"/>
-        <v>499</v>
+        <v>1399</v>
       </c>
       <c r="H8">
         <f t="shared" si="1"/>
-        <v>9.98</v>
+        <v>27.98</v>
       </c>
       <c r="I8">
         <f t="shared" si="2"/>
-        <v>489.02</v>
+        <v>1371.02</v>
       </c>
       <c r="J8">
         <f t="shared" si="3"/>
-        <v>339.02</v>
+        <v>651.02</v>
       </c>
       <c r="K8" s="1">
         <f t="shared" si="4"/>
-        <v>0.6793987975951904</v>
+        <v>0.46534667619728376</v>
       </c>
       <c r="L8" t="str">
         <f t="shared" si="5"/>
-        <v>₹499</v>
+        <v>₹1,399</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
@@ -1334,27 +1343,27 @@
       </c>
       <c r="G9">
         <f t="shared" si="6"/>
-        <v>499</v>
+        <v>399</v>
       </c>
       <c r="H9">
         <f t="shared" si="1"/>
-        <v>9.98</v>
+        <v>7.98</v>
       </c>
       <c r="I9">
         <f t="shared" si="2"/>
-        <v>489.02</v>
+        <v>391.02</v>
       </c>
       <c r="J9">
         <f t="shared" si="3"/>
-        <v>339.02</v>
+        <v>241.01999999999998</v>
       </c>
       <c r="K9" s="1">
         <f t="shared" si="4"/>
-        <v>0.6793987975951904</v>
+        <v>0.60406015037593985</v>
       </c>
       <c r="L9" t="str">
         <f t="shared" si="5"/>
-        <v>₹499</v>
+        <v>₹399</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
@@ -1373,27 +1382,27 @@
       </c>
       <c r="G10">
         <f t="shared" si="6"/>
-        <v>499</v>
+        <v>599</v>
       </c>
       <c r="H10">
         <f t="shared" si="1"/>
-        <v>9.98</v>
+        <v>11.98</v>
       </c>
       <c r="I10">
         <f t="shared" si="2"/>
-        <v>489.02</v>
+        <v>587.02</v>
       </c>
       <c r="J10">
         <f t="shared" si="3"/>
-        <v>339.02</v>
+        <v>437.02</v>
       </c>
       <c r="K10" s="1">
         <f t="shared" si="4"/>
-        <v>0.6793987975951904</v>
+        <v>0.72958263772954923</v>
       </c>
       <c r="L10" t="str">
         <f t="shared" si="5"/>
-        <v>₹499</v>
+        <v>₹599</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
@@ -1412,27 +1421,27 @@
       </c>
       <c r="G11">
         <f t="shared" si="6"/>
-        <v>499</v>
+        <v>599</v>
       </c>
       <c r="H11">
         <f t="shared" si="1"/>
-        <v>9.98</v>
+        <v>11.98</v>
       </c>
       <c r="I11">
         <f t="shared" si="2"/>
-        <v>489.02</v>
+        <v>587.02</v>
       </c>
       <c r="J11">
         <f t="shared" si="3"/>
-        <v>339.02</v>
+        <v>437.02</v>
       </c>
       <c r="K11" s="1">
         <f t="shared" si="4"/>
-        <v>0.6793987975951904</v>
+        <v>0.72958263772954923</v>
       </c>
       <c r="L11" t="str">
         <f t="shared" si="5"/>
-        <v>₹499</v>
+        <v>₹599</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
@@ -1451,27 +1460,27 @@
       </c>
       <c r="G12">
         <f t="shared" si="6"/>
-        <v>499</v>
+        <v>399</v>
       </c>
       <c r="H12">
         <f t="shared" si="1"/>
-        <v>9.98</v>
+        <v>7.98</v>
       </c>
       <c r="I12">
         <f t="shared" si="2"/>
-        <v>489.02</v>
+        <v>391.02</v>
       </c>
       <c r="J12">
         <f t="shared" si="3"/>
-        <v>359.02</v>
+        <v>261.02</v>
       </c>
       <c r="K12" s="1">
         <f t="shared" si="4"/>
-        <v>0.71947895791583161</v>
+        <v>0.65418546365914787</v>
       </c>
       <c r="L12" t="str">
         <f t="shared" si="5"/>
-        <v>₹499</v>
+        <v>₹399</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
@@ -1490,27 +1499,27 @@
       </c>
       <c r="G13">
         <f t="shared" si="6"/>
-        <v>499</v>
+        <v>399</v>
       </c>
       <c r="H13">
         <f t="shared" si="1"/>
-        <v>9.98</v>
+        <v>7.98</v>
       </c>
       <c r="I13">
         <f t="shared" si="2"/>
-        <v>489.02</v>
+        <v>391.02</v>
       </c>
       <c r="J13">
         <f t="shared" si="3"/>
-        <v>359.02</v>
+        <v>261.02</v>
       </c>
       <c r="K13" s="1">
         <f t="shared" si="4"/>
-        <v>0.71947895791583161</v>
+        <v>0.65418546365914787</v>
       </c>
       <c r="L13" t="str">
         <f t="shared" si="5"/>
-        <v>₹499</v>
+        <v>₹399</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
@@ -1529,27 +1538,27 @@
       </c>
       <c r="G14">
         <f t="shared" si="6"/>
-        <v>499</v>
+        <v>599</v>
       </c>
       <c r="H14">
         <f t="shared" si="1"/>
-        <v>9.98</v>
+        <v>11.98</v>
       </c>
       <c r="I14">
         <f t="shared" si="2"/>
-        <v>489.02</v>
+        <v>587.02</v>
       </c>
       <c r="J14">
         <f t="shared" si="3"/>
-        <v>339.02</v>
+        <v>437.02</v>
       </c>
       <c r="K14" s="1">
         <f t="shared" si="4"/>
-        <v>0.6793987975951904</v>
+        <v>0.72958263772954923</v>
       </c>
       <c r="L14" t="str">
         <f t="shared" si="5"/>
-        <v>₹499</v>
+        <v>₹599</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
@@ -1568,27 +1577,27 @@
       </c>
       <c r="G15">
         <f t="shared" si="6"/>
-        <v>499</v>
+        <v>599</v>
       </c>
       <c r="H15">
         <f t="shared" si="1"/>
-        <v>9.98</v>
+        <v>11.98</v>
       </c>
       <c r="I15">
         <f t="shared" si="2"/>
-        <v>489.02</v>
+        <v>587.02</v>
       </c>
       <c r="J15">
         <f t="shared" si="3"/>
-        <v>339.02</v>
+        <v>437.02</v>
       </c>
       <c r="K15" s="1">
         <f t="shared" si="4"/>
-        <v>0.6793987975951904</v>
+        <v>0.72958263772954923</v>
       </c>
       <c r="L15" t="str">
         <f t="shared" si="5"/>
-        <v>₹499</v>
+        <v>₹599</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
@@ -1607,27 +1616,27 @@
       </c>
       <c r="G16">
         <f t="shared" si="6"/>
-        <v>499</v>
+        <v>599</v>
       </c>
       <c r="H16">
         <f t="shared" si="1"/>
-        <v>9.98</v>
+        <v>11.98</v>
       </c>
       <c r="I16">
         <f t="shared" si="2"/>
-        <v>489.02</v>
+        <v>587.02</v>
       </c>
       <c r="J16">
         <f t="shared" si="3"/>
-        <v>339.02</v>
+        <v>437.02</v>
       </c>
       <c r="K16" s="1">
         <f t="shared" si="4"/>
-        <v>0.6793987975951904</v>
+        <v>0.72958263772954923</v>
       </c>
       <c r="L16" t="str">
         <f t="shared" si="5"/>
-        <v>₹499</v>
+        <v>₹599</v>
       </c>
     </row>
     <row r="17" spans="3:12" x14ac:dyDescent="0.3">
@@ -1646,27 +1655,27 @@
       </c>
       <c r="G17">
         <f t="shared" si="6"/>
-        <v>499</v>
+        <v>599</v>
       </c>
       <c r="H17">
         <f t="shared" si="1"/>
-        <v>9.98</v>
+        <v>11.98</v>
       </c>
       <c r="I17">
         <f t="shared" si="2"/>
-        <v>489.02</v>
+        <v>587.02</v>
       </c>
       <c r="J17">
         <f t="shared" si="3"/>
-        <v>339.02</v>
+        <v>437.02</v>
       </c>
       <c r="K17" s="1">
         <f t="shared" si="4"/>
-        <v>0.6793987975951904</v>
+        <v>0.72958263772954923</v>
       </c>
       <c r="L17" t="str">
         <f t="shared" si="5"/>
-        <v>₹499</v>
+        <v>₹599</v>
       </c>
     </row>
     <row r="18" spans="3:12" x14ac:dyDescent="0.3">
@@ -1684,28 +1693,28 @@
         <v>3</v>
       </c>
       <c r="G18">
-        <f t="shared" ref="G18" si="8">ROUNDUP((E18*F18)/500,0)*500-1</f>
-        <v>499</v>
+        <f t="shared" si="6"/>
+        <v>599</v>
       </c>
       <c r="H18">
         <f t="shared" si="1"/>
-        <v>9.98</v>
+        <v>11.98</v>
       </c>
       <c r="I18">
-        <f t="shared" ref="I18" si="9">G18-H18</f>
-        <v>489.02</v>
+        <f t="shared" ref="I18" si="8">G18-H18</f>
+        <v>587.02</v>
       </c>
       <c r="J18">
-        <f t="shared" ref="J18" si="10">I18-E18</f>
-        <v>339.02</v>
+        <f t="shared" ref="J18" si="9">I18-E18</f>
+        <v>437.02</v>
       </c>
       <c r="K18" s="1">
-        <f t="shared" ref="K18" si="11">J18/G18</f>
-        <v>0.6793987975951904</v>
+        <f t="shared" ref="K18" si="10">J18/G18</f>
+        <v>0.72958263772954923</v>
       </c>
       <c r="L18" t="str">
-        <f t="shared" ref="L18" si="12">"₹"&amp;TEXT(G18,"#,##0")</f>
-        <v>₹499</v>
+        <f t="shared" ref="L18" si="11">"₹"&amp;TEXT(G18,"#,##0")</f>
+        <v>₹599</v>
       </c>
     </row>
   </sheetData>

</xml_diff>